<commit_message>
Atualização da planilha modelo
</commit_message>
<xml_diff>
--- a/public/assets/template_importacao_bens.xlsx
+++ b/public/assets/template_importacao_bens.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importacao" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -36,7 +36,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -46,6 +46,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002F7D57"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F5EE"/>
       </patternFill>
     </fill>
   </fills>
@@ -75,13 +80,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -448,82 +456,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="35" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>numero_patrimonial</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>nome</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>nome</t>
+          <t>descricao</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>marca</t>
+          <t>valor_unitario</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>modelo</t>
+          <t>marca</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>descricao</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>valor_unitario</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>numero_processo</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>numero_patrimonial</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>localizacao</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>criado_por__nome</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>criado_em</t>
+          <t>modelo</t>
         </is>
       </c>
     </row>
@@ -534,26 +506,14 @@
       <c r="D2" s="2" t="n"/>
       <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="n"/>
-      <c r="L2" s="2" t="n"/>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="2" t="n"/>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="n"/>
-      <c r="I3" s="2" t="n"/>
-      <c r="J3" s="2" t="n"/>
-      <c r="K3" s="2" t="n"/>
-      <c r="L3" s="2" t="n"/>
+      <c r="A3" s="3" t="n"/>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n"/>
+      <c r="F3" s="3" t="n"/>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="2" t="n"/>
@@ -562,26 +522,14 @@
       <c r="D4" s="2" t="n"/>
       <c r="E4" s="2" t="n"/>
       <c r="F4" s="2" t="n"/>
-      <c r="G4" s="2" t="n"/>
-      <c r="H4" s="2" t="n"/>
-      <c r="I4" s="2" t="n"/>
-      <c r="J4" s="2" t="n"/>
-      <c r="K4" s="2" t="n"/>
-      <c r="L4" s="2" t="n"/>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="2" t="n"/>
-      <c r="B5" s="2" t="n"/>
-      <c r="C5" s="2" t="n"/>
-      <c r="D5" s="2" t="n"/>
-      <c r="E5" s="2" t="n"/>
-      <c r="F5" s="2" t="n"/>
-      <c r="G5" s="2" t="n"/>
-      <c r="H5" s="2" t="n"/>
-      <c r="I5" s="2" t="n"/>
-      <c r="J5" s="2" t="n"/>
-      <c r="K5" s="2" t="n"/>
-      <c r="L5" s="2" t="n"/>
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="3" t="n"/>
+      <c r="C5" s="3" t="n"/>
+      <c r="D5" s="3" t="n"/>
+      <c r="E5" s="3" t="n"/>
+      <c r="F5" s="3" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="2" t="n"/>
@@ -590,26 +538,14 @@
       <c r="D6" s="2" t="n"/>
       <c r="E6" s="2" t="n"/>
       <c r="F6" s="2" t="n"/>
-      <c r="G6" s="2" t="n"/>
-      <c r="H6" s="2" t="n"/>
-      <c r="I6" s="2" t="n"/>
-      <c r="J6" s="2" t="n"/>
-      <c r="K6" s="2" t="n"/>
-      <c r="L6" s="2" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="2" t="n"/>
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="n"/>
-      <c r="I7" s="2" t="n"/>
-      <c r="J7" s="2" t="n"/>
-      <c r="K7" s="2" t="n"/>
-      <c r="L7" s="2" t="n"/>
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="3" t="n"/>
+      <c r="C7" s="3" t="n"/>
+      <c r="D7" s="3" t="n"/>
+      <c r="E7" s="3" t="n"/>
+      <c r="F7" s="3" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="2" t="n"/>
@@ -618,26 +554,14 @@
       <c r="D8" s="2" t="n"/>
       <c r="E8" s="2" t="n"/>
       <c r="F8" s="2" t="n"/>
-      <c r="G8" s="2" t="n"/>
-      <c r="H8" s="2" t="n"/>
-      <c r="I8" s="2" t="n"/>
-      <c r="J8" s="2" t="n"/>
-      <c r="K8" s="2" t="n"/>
-      <c r="L8" s="2" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="2" t="n"/>
-      <c r="B9" s="2" t="n"/>
-      <c r="C9" s="2" t="n"/>
-      <c r="D9" s="2" t="n"/>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="2" t="n"/>
-      <c r="G9" s="2" t="n"/>
-      <c r="H9" s="2" t="n"/>
-      <c r="I9" s="2" t="n"/>
-      <c r="J9" s="2" t="n"/>
-      <c r="K9" s="2" t="n"/>
-      <c r="L9" s="2" t="n"/>
+      <c r="A9" s="3" t="n"/>
+      <c r="B9" s="3" t="n"/>
+      <c r="C9" s="3" t="n"/>
+      <c r="D9" s="3" t="n"/>
+      <c r="E9" s="3" t="n"/>
+      <c r="F9" s="3" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="2" t="n"/>
@@ -646,26 +570,14 @@
       <c r="D10" s="2" t="n"/>
       <c r="E10" s="2" t="n"/>
       <c r="F10" s="2" t="n"/>
-      <c r="G10" s="2" t="n"/>
-      <c r="H10" s="2" t="n"/>
-      <c r="I10" s="2" t="n"/>
-      <c r="J10" s="2" t="n"/>
-      <c r="K10" s="2" t="n"/>
-      <c r="L10" s="2" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="2" t="n"/>
-      <c r="B11" s="2" t="n"/>
-      <c r="C11" s="2" t="n"/>
-      <c r="D11" s="2" t="n"/>
-      <c r="E11" s="2" t="n"/>
-      <c r="F11" s="2" t="n"/>
-      <c r="G11" s="2" t="n"/>
-      <c r="H11" s="2" t="n"/>
-      <c r="I11" s="2" t="n"/>
-      <c r="J11" s="2" t="n"/>
-      <c r="K11" s="2" t="n"/>
-      <c r="L11" s="2" t="n"/>
+      <c r="A11" s="3" t="n"/>
+      <c r="B11" s="3" t="n"/>
+      <c r="C11" s="3" t="n"/>
+      <c r="D11" s="3" t="n"/>
+      <c r="E11" s="3" t="n"/>
+      <c r="F11" s="3" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="2" t="n"/>
@@ -674,26 +586,14 @@
       <c r="D12" s="2" t="n"/>
       <c r="E12" s="2" t="n"/>
       <c r="F12" s="2" t="n"/>
-      <c r="G12" s="2" t="n"/>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="n"/>
-      <c r="J12" s="2" t="n"/>
-      <c r="K12" s="2" t="n"/>
-      <c r="L12" s="2" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="2" t="n"/>
-      <c r="B13" s="2" t="n"/>
-      <c r="C13" s="2" t="n"/>
-      <c r="D13" s="2" t="n"/>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="n"/>
-      <c r="G13" s="2" t="n"/>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="n"/>
-      <c r="J13" s="2" t="n"/>
-      <c r="K13" s="2" t="n"/>
-      <c r="L13" s="2" t="n"/>
+      <c r="A13" s="3" t="n"/>
+      <c r="B13" s="3" t="n"/>
+      <c r="C13" s="3" t="n"/>
+      <c r="D13" s="3" t="n"/>
+      <c r="E13" s="3" t="n"/>
+      <c r="F13" s="3" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="2" t="n"/>
@@ -702,26 +602,14 @@
       <c r="D14" s="2" t="n"/>
       <c r="E14" s="2" t="n"/>
       <c r="F14" s="2" t="n"/>
-      <c r="G14" s="2" t="n"/>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="n"/>
-      <c r="J14" s="2" t="n"/>
-      <c r="K14" s="2" t="n"/>
-      <c r="L14" s="2" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="2" t="n"/>
-      <c r="B15" s="2" t="n"/>
-      <c r="C15" s="2" t="n"/>
-      <c r="D15" s="2" t="n"/>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="2" t="n"/>
-      <c r="G15" s="2" t="n"/>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="n"/>
-      <c r="J15" s="2" t="n"/>
-      <c r="K15" s="2" t="n"/>
-      <c r="L15" s="2" t="n"/>
+      <c r="A15" s="3" t="n"/>
+      <c r="B15" s="3" t="n"/>
+      <c r="C15" s="3" t="n"/>
+      <c r="D15" s="3" t="n"/>
+      <c r="E15" s="3" t="n"/>
+      <c r="F15" s="3" t="n"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="2" t="n"/>
@@ -730,26 +618,14 @@
       <c r="D16" s="2" t="n"/>
       <c r="E16" s="2" t="n"/>
       <c r="F16" s="2" t="n"/>
-      <c r="G16" s="2" t="n"/>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="n"/>
-      <c r="J16" s="2" t="n"/>
-      <c r="K16" s="2" t="n"/>
-      <c r="L16" s="2" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="2" t="n"/>
-      <c r="B17" s="2" t="n"/>
-      <c r="C17" s="2" t="n"/>
-      <c r="D17" s="2" t="n"/>
-      <c r="E17" s="2" t="n"/>
-      <c r="F17" s="2" t="n"/>
-      <c r="G17" s="2" t="n"/>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="n"/>
-      <c r="J17" s="2" t="n"/>
-      <c r="K17" s="2" t="n"/>
-      <c r="L17" s="2" t="n"/>
+      <c r="A17" s="3" t="n"/>
+      <c r="B17" s="3" t="n"/>
+      <c r="C17" s="3" t="n"/>
+      <c r="D17" s="3" t="n"/>
+      <c r="E17" s="3" t="n"/>
+      <c r="F17" s="3" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="2" t="n"/>
@@ -758,26 +634,14 @@
       <c r="D18" s="2" t="n"/>
       <c r="E18" s="2" t="n"/>
       <c r="F18" s="2" t="n"/>
-      <c r="G18" s="2" t="n"/>
-      <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="n"/>
-      <c r="J18" s="2" t="n"/>
-      <c r="K18" s="2" t="n"/>
-      <c r="L18" s="2" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="2" t="n"/>
-      <c r="B19" s="2" t="n"/>
-      <c r="C19" s="2" t="n"/>
-      <c r="D19" s="2" t="n"/>
-      <c r="E19" s="2" t="n"/>
-      <c r="F19" s="2" t="n"/>
-      <c r="G19" s="2" t="n"/>
-      <c r="H19" s="2" t="n"/>
-      <c r="I19" s="2" t="n"/>
-      <c r="J19" s="2" t="n"/>
-      <c r="K19" s="2" t="n"/>
-      <c r="L19" s="2" t="n"/>
+      <c r="A19" s="3" t="n"/>
+      <c r="B19" s="3" t="n"/>
+      <c r="C19" s="3" t="n"/>
+      <c r="D19" s="3" t="n"/>
+      <c r="E19" s="3" t="n"/>
+      <c r="F19" s="3" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="2" t="n"/>
@@ -786,26 +650,14 @@
       <c r="D20" s="2" t="n"/>
       <c r="E20" s="2" t="n"/>
       <c r="F20" s="2" t="n"/>
-      <c r="G20" s="2" t="n"/>
-      <c r="H20" s="2" t="n"/>
-      <c r="I20" s="2" t="n"/>
-      <c r="J20" s="2" t="n"/>
-      <c r="K20" s="2" t="n"/>
-      <c r="L20" s="2" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="2" t="n"/>
-      <c r="B21" s="2" t="n"/>
-      <c r="C21" s="2" t="n"/>
-      <c r="D21" s="2" t="n"/>
-      <c r="E21" s="2" t="n"/>
-      <c r="F21" s="2" t="n"/>
-      <c r="G21" s="2" t="n"/>
-      <c r="H21" s="2" t="n"/>
-      <c r="I21" s="2" t="n"/>
-      <c r="J21" s="2" t="n"/>
-      <c r="K21" s="2" t="n"/>
-      <c r="L21" s="2" t="n"/>
+      <c r="A21" s="3" t="n"/>
+      <c r="B21" s="3" t="n"/>
+      <c r="C21" s="3" t="n"/>
+      <c r="D21" s="3" t="n"/>
+      <c r="E21" s="3" t="n"/>
+      <c r="F21" s="3" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="2" t="n"/>
@@ -814,26 +666,14 @@
       <c r="D22" s="2" t="n"/>
       <c r="E22" s="2" t="n"/>
       <c r="F22" s="2" t="n"/>
-      <c r="G22" s="2" t="n"/>
-      <c r="H22" s="2" t="n"/>
-      <c r="I22" s="2" t="n"/>
-      <c r="J22" s="2" t="n"/>
-      <c r="K22" s="2" t="n"/>
-      <c r="L22" s="2" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="2" t="n"/>
-      <c r="B23" s="2" t="n"/>
-      <c r="C23" s="2" t="n"/>
-      <c r="D23" s="2" t="n"/>
-      <c r="E23" s="2" t="n"/>
-      <c r="F23" s="2" t="n"/>
-      <c r="G23" s="2" t="n"/>
-      <c r="H23" s="2" t="n"/>
-      <c r="I23" s="2" t="n"/>
-      <c r="J23" s="2" t="n"/>
-      <c r="K23" s="2" t="n"/>
-      <c r="L23" s="2" t="n"/>
+      <c r="A23" s="3" t="n"/>
+      <c r="B23" s="3" t="n"/>
+      <c r="C23" s="3" t="n"/>
+      <c r="D23" s="3" t="n"/>
+      <c r="E23" s="3" t="n"/>
+      <c r="F23" s="3" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="2" t="n"/>
@@ -842,26 +682,14 @@
       <c r="D24" s="2" t="n"/>
       <c r="E24" s="2" t="n"/>
       <c r="F24" s="2" t="n"/>
-      <c r="G24" s="2" t="n"/>
-      <c r="H24" s="2" t="n"/>
-      <c r="I24" s="2" t="n"/>
-      <c r="J24" s="2" t="n"/>
-      <c r="K24" s="2" t="n"/>
-      <c r="L24" s="2" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="2" t="n"/>
-      <c r="B25" s="2" t="n"/>
-      <c r="C25" s="2" t="n"/>
-      <c r="D25" s="2" t="n"/>
-      <c r="E25" s="2" t="n"/>
-      <c r="F25" s="2" t="n"/>
-      <c r="G25" s="2" t="n"/>
-      <c r="H25" s="2" t="n"/>
-      <c r="I25" s="2" t="n"/>
-      <c r="J25" s="2" t="n"/>
-      <c r="K25" s="2" t="n"/>
-      <c r="L25" s="2" t="n"/>
+      <c r="A25" s="3" t="n"/>
+      <c r="B25" s="3" t="n"/>
+      <c r="C25" s="3" t="n"/>
+      <c r="D25" s="3" t="n"/>
+      <c r="E25" s="3" t="n"/>
+      <c r="F25" s="3" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="2" t="n"/>
@@ -870,26 +698,14 @@
       <c r="D26" s="2" t="n"/>
       <c r="E26" s="2" t="n"/>
       <c r="F26" s="2" t="n"/>
-      <c r="G26" s="2" t="n"/>
-      <c r="H26" s="2" t="n"/>
-      <c r="I26" s="2" t="n"/>
-      <c r="J26" s="2" t="n"/>
-      <c r="K26" s="2" t="n"/>
-      <c r="L26" s="2" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="2" t="n"/>
-      <c r="B27" s="2" t="n"/>
-      <c r="C27" s="2" t="n"/>
-      <c r="D27" s="2" t="n"/>
-      <c r="E27" s="2" t="n"/>
-      <c r="F27" s="2" t="n"/>
-      <c r="G27" s="2" t="n"/>
-      <c r="H27" s="2" t="n"/>
-      <c r="I27" s="2" t="n"/>
-      <c r="J27" s="2" t="n"/>
-      <c r="K27" s="2" t="n"/>
-      <c r="L27" s="2" t="n"/>
+      <c r="A27" s="3" t="n"/>
+      <c r="B27" s="3" t="n"/>
+      <c r="C27" s="3" t="n"/>
+      <c r="D27" s="3" t="n"/>
+      <c r="E27" s="3" t="n"/>
+      <c r="F27" s="3" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="2" t="n"/>
@@ -898,26 +714,14 @@
       <c r="D28" s="2" t="n"/>
       <c r="E28" s="2" t="n"/>
       <c r="F28" s="2" t="n"/>
-      <c r="G28" s="2" t="n"/>
-      <c r="H28" s="2" t="n"/>
-      <c r="I28" s="2" t="n"/>
-      <c r="J28" s="2" t="n"/>
-      <c r="K28" s="2" t="n"/>
-      <c r="L28" s="2" t="n"/>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="2" t="n"/>
-      <c r="B29" s="2" t="n"/>
-      <c r="C29" s="2" t="n"/>
-      <c r="D29" s="2" t="n"/>
-      <c r="E29" s="2" t="n"/>
-      <c r="F29" s="2" t="n"/>
-      <c r="G29" s="2" t="n"/>
-      <c r="H29" s="2" t="n"/>
-      <c r="I29" s="2" t="n"/>
-      <c r="J29" s="2" t="n"/>
-      <c r="K29" s="2" t="n"/>
-      <c r="L29" s="2" t="n"/>
+      <c r="A29" s="3" t="n"/>
+      <c r="B29" s="3" t="n"/>
+      <c r="C29" s="3" t="n"/>
+      <c r="D29" s="3" t="n"/>
+      <c r="E29" s="3" t="n"/>
+      <c r="F29" s="3" t="n"/>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="2" t="n"/>
@@ -926,33 +730,16 @@
       <c r="D30" s="2" t="n"/>
       <c r="E30" s="2" t="n"/>
       <c r="F30" s="2" t="n"/>
-      <c r="G30" s="2" t="n"/>
-      <c r="H30" s="2" t="n"/>
-      <c r="I30" s="2" t="n"/>
-      <c r="J30" s="2" t="n"/>
-      <c r="K30" s="2" t="n"/>
-      <c r="L30" s="2" t="n"/>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="2" t="n"/>
-      <c r="B31" s="2" t="n"/>
-      <c r="C31" s="2" t="n"/>
-      <c r="D31" s="2" t="n"/>
-      <c r="E31" s="2" t="n"/>
-      <c r="F31" s="2" t="n"/>
-      <c r="G31" s="2" t="n"/>
-      <c r="H31" s="2" t="n"/>
-      <c r="I31" s="2" t="n"/>
-      <c r="J31" s="2" t="n"/>
-      <c r="K31" s="2" t="n"/>
-      <c r="L31" s="2" t="n"/>
+      <c r="A31" s="3" t="n"/>
+      <c r="B31" s="3" t="n"/>
+      <c r="C31" s="3" t="n"/>
+      <c r="D31" s="3" t="n"/>
+      <c r="E31" s="3" t="n"/>
+      <c r="F31" s="3" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="B2:B31" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Status inválido" error="Valor inválido. Escolha um da lista." type="list">
-      <formula1>"aguardando_aprovacao,aprovado,nao_aprovado,baixa_fisica"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>